<commit_message>
feat(F-NAR-008): 3 histoires réécrites (Lina, Noé, Tom)
Fil rouge : petit soleil, carotte du marché, bateau-chaise.
Début et fin vécus. Leçon greffée, pas un cours.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
+++ b/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La petite tomate de Lina</t>
+          <t>Le petit soleil dans l'assiette</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Lina veut savoir si la tomate, brillante comme un petit soleil dans l'assiette, a vraiment le goût du soleil.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>C'est l'heure du déjeuner. Lina s'assoit à table, près de maman. Dans l'assiette, il y a du riz, et une petite tomate rouge. Lina regarde la tomate. Elle est ronde. Elle sent le jardin. Maman sourit. Tu peux goûter une petite bouchée. Juste une petite bouchée. Lina prend un tout petit morceau. Elle le met dans sa bouche. C'est doux. C'est un peu juteux. C'est doux, maman. Merci d'avoir goûté. Tu as su nommer le goût. Une petite portion, c'est déjà bien.</t>
+          <t>Lina pousse la porte de la cuisine. Le soleil entre avec elle. Maman est là, près de la table. Maman, le soleil est tout jaune ! Viens, Lina. L'assiette est prête. Lina s'assoit tout près de maman. Dans l'assiette, une petite tomate. Elle est ronde. Elle est rouge. Elle brille. C'est un petit soleil ! Un petit soleil dans l'assiette. Lina se penche tout près. Ça sent le jardin. Il a le goût du soleil ? Tu peux goûter une petite bouchée. Juste une petite portion. Lina prend un tout petit morceau. Elle le met dans sa bouche. C'est doux. C'est un peu juteux. C'est doux, maman. Un peu sucré. Doux et sucré. Comme un soleil. Lina a nommé le goût. Le petit soleil reste dans l'assiette. Lina a trouvé le goût.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1240,7 +1252,7 @@
         <v>0.86</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1312,15 +1324,31 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|C'est l'heure du déjeuner. Lina s'assoit à table, près de maman. Dans l'assiette, il y a du riz, et une petite tomate rouge. Lina regarde la tomate. Elle est ronde. Elle sent le jardin. Maman sourit.
-maman|Tu peux goûter une petite bouchée. Juste une petite bouchée.
-narrateur|Lina prend un tout petit morceau. Elle le met dans sa bouche. C'est doux. C'est un peu juteux.
-enfant-f|C'est doux, maman.
-maman|Merci d'avoir goûté. Tu as su nommer le goût.
-narrateur|Une petite portion, c'est déjà bien.</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr"/>
+          <t>narrateur|Lina pousse la porte de la cuisine.
+narrateur|Le soleil entre avec elle.
+narrateur|Maman est là, près de la table.
+enfant-f|Maman, le soleil est tout jaune !
+maman|Viens, Lina. L'assiette est prête.
+narrateur|Lina s'assoit tout près de maman.
+narrateur|Dans l'assiette, une petite tomate.
+narrateur|Elle est ronde. Elle est rouge. Elle brille.
+enfant-f|C'est un petit soleil !
+maman|Un petit soleil dans l'assiette.
+narrateur|Lina se penche tout près.
+narrateur|Ça sent le jardin.
+enfant-f|Il a le goût du soleil ?
+maman|Tu peux goûter une petite bouchée.
+narrateur|Juste une petite portion.
+narrateur|Lina prend un tout petit morceau.
+narrateur|Elle le met dans sa bouche.
+narrateur|C'est doux. C'est un peu juteux.
+enfant-f|C'est doux, maman. Un peu sucré.
+maman|Doux et sucré. Comme un soleil.
+narrateur|Lina a nommé le goût.
+narrateur|Le petit soleil reste dans l'assiette.
+narrateur|Lina a trouvé le goût.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1345,7 +1373,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Lina goûte la tomate. Que fait-elle ?</t>
+          <t>Lina veut le goût du petit soleil. Que fait-elle ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1429,7 +1457,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,10 +1529,9 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Lina goûte la tomate. Que fait-elle ?</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr"/>
+          <t>narrateur|Lina veut le goût du petit soleil. Que fait-elle ?</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1529,7 +1556,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lina a goûté. Elle a nommé le goût. Maman est là. Une petite portion, c'est assez.</t>
+          <t>Lina a goûté. Elle a su nommer le goût. Une petite portion, c'est assez. Maman est là.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1597,7 +1624,7 @@
         <v>0.86</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,10 +1700,12 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Lina a goûté. Elle a nommé le goût. Maman est là. Une petite portion, c'est assez.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+          <t>narrateur|Lina a goûté.
+narrateur|Elle a su nommer le goût.
+narrateur|Une petite portion, c'est assez.
+narrateur|Maman est là.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1701,7 +1730,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Lina boit une gorgée d'eau. La tomate reste dans l'assiette, à sa place. Lina dit merci.</t>
+          <t>Lina boit une gorgée d'eau. Le petit soleil reste dans l'assiette. Merci, maman. Merci d'avoir goûté.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1769,7 +1798,7 @@
         <v>0.86</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.2</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1837,10 +1866,12 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Lina boit une gorgée d'eau. La tomate reste dans l'assiette, à sa place. Lina dit merci.</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr"/>
+          <t>narrateur|Lina boit une gorgée d'eau.
+narrateur|Le petit soleil reste dans l'assiette.
+enfant-f|Merci, maman.
+maman|Merci d'avoir goûté.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1865,7 +1896,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Dans la cuisine, le soleil brille encore. Il était doux, le petit soleil. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1933,7 +1964,7 @@
         <v>0.82</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.36</v>
+        <v>1.2</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2005,10 +2036,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr"/>
+          <t>narrateur|Dans la cuisine, le soleil brille encore.
+enfant-f|Il était doux, le petit soleil.
+narrateur|L'histoire est finie.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2027,7 +2059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2065,6 +2097,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit captivant, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-008): passe 2 — Lina, Noé, Tom pour 3–6 ans
Fusion éditoriale des agents C/D : un fil par histoire, un moment
par chunk, phrases N1/N2, leçon vécue en fin. L’ancienne version
passe 1 est remplacée dans les arbres (classroom conservé en original.xlsx).
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
+++ b/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lina veut savoir si la tomate, brillante comme un petit soleil dans l'assiette, a vraiment le goût du soleil.</t>
+          <t>Lina a faim. Une tomate rouge brille dans son assiette, comme un petit soleil. Elle en goûte une petite bouchée.</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lina pousse la porte de la cuisine. Le soleil entre avec elle. Maman est là, près de la table. Maman, le soleil est tout jaune ! Viens, Lina. L'assiette est prête. Lina s'assoit tout près de maman. Dans l'assiette, une petite tomate. Elle est ronde. Elle est rouge. Elle brille. C'est un petit soleil ! Un petit soleil dans l'assiette. Lina se penche tout près. Ça sent le jardin. Il a le goût du soleil ? Tu peux goûter une petite bouchée. Juste une petite portion. Lina prend un tout petit morceau. Elle le met dans sa bouche. C'est doux. C'est un peu juteux. C'est doux, maman. Un peu sucré. Doux et sucré. Comme un soleil. Lina a nommé le goût. Le petit soleil reste dans l'assiette. Lina a trouvé le goût.</t>
+          <t>Lina entre dans la cuisine. Il y a du soleil. Maman est près de la table. Maman, j'ai faim ! Viens, Lina. Ton assiette est là. Lina s'assoit près de maman. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille. C'est un petit soleil ! Oui, un petit soleil. Lina se penche tout près. Ça sent le jardin. Il a quel goût ? Tu peux goûter. Une petite bouchée. Lina prend une petite bouchée. Elle goûte.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
         <v>0.86</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.2</v>
+        <v>1.32</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1324,29 +1324,31 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Lina pousse la porte de la cuisine.
-narrateur|Le soleil entre avec elle.
-narrateur|Maman est là, près de la table.
-enfant-f|Maman, le soleil est tout jaune !
-maman|Viens, Lina. L'assiette est prête.
-narrateur|Lina s'assoit tout près de maman.
-narrateur|Dans l'assiette, une petite tomate.
-narrateur|Elle est ronde. Elle est rouge. Elle brille.
+          <t>narrateur|Lina entre dans la cuisine.
+narrateur|Il y a du soleil.
+narrateur|Maman est près de la table.
+enfant-f|Maman, j'ai faim !
+maman|Viens, Lina.
+maman|Ton assiette est là.
+narrateur|Lina s'assoit près de maman.
+narrateur|Dans l'assiette, une tomate.
+narrateur|Elle est ronde.
+narrateur|Elle est rouge.
+narrateur|Elle brille.
 enfant-f|C'est un petit soleil !
-maman|Un petit soleil dans l'assiette.
+maman|Oui, un petit soleil.
 narrateur|Lina se penche tout près.
 narrateur|Ça sent le jardin.
-enfant-f|Il a le goût du soleil ?
-maman|Tu peux goûter une petite bouchée.
-narrateur|Juste une petite portion.
-narrateur|Lina prend un tout petit morceau.
-narrateur|Elle le met dans sa bouche.
-narrateur|C'est doux. C'est un peu juteux.
-enfant-f|C'est doux, maman. Un peu sucré.
-maman|Doux et sucré. Comme un soleil.
-narrateur|Lina a nommé le goût.
-narrateur|Le petit soleil reste dans l'assiette.
-narrateur|Lina a trouvé le goût.</t>
+enfant-f|Il a quel goût ?
+maman|Tu peux goûter.
+maman|Une petite bouchée.
+narrateur|Lina prend une petite bouchée.
+narrateur|Elle goûte.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>porte</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1375,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Lina veut le goût du petit soleil. Que fait-elle ?</t>
+          <t>Que fait Lina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1457,7 +1459,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1529,9 +1531,10 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Lina veut le goût du petit soleil. Que fait-elle ?</t>
-        </is>
-      </c>
+          <t>narrateur|Que fait Lina ?</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1556,7 +1559,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lina a goûté. Elle a su nommer le goût. Une petite portion, c'est assez. Maman est là.</t>
+          <t>Lina mâche. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Le petit soleil est encore là.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1624,7 +1627,7 @@
         <v>0.86</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1700,12 +1703,16 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Lina a goûté.
-narrateur|Elle a su nommer le goût.
-narrateur|Une petite portion, c'est assez.
-narrateur|Maman est là.</t>
-        </is>
-      </c>
+          <t>narrateur|Lina mâche.
+enfant-f|C'est doux, maman.
+enfant-f|Un peu sucré.
+enfant-f|Comme un soleil.
+maman|Oui.
+maman|Doux et sucré.
+narrateur|Le petit soleil est encore là.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1730,7 +1737,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Lina boit une gorgée d'eau. Le petit soleil reste dans l'assiette. Merci, maman. Merci d'avoir goûté.</t>
+          <t>Lina boit une gorgée d'eau. Le petit soleil reste dans l'assiette. Merci, maman. Merci, Lina.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1798,7 +1805,7 @@
         <v>0.86</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1869,9 +1876,10 @@
           <t>narrateur|Lina boit une gorgée d'eau.
 narrateur|Le petit soleil reste dans l'assiette.
 enfant-f|Merci, maman.
-maman|Merci d'avoir goûté.</t>
-        </is>
-      </c>
+maman|Merci, Lina.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1896,7 +1904,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Dans la cuisine, le soleil brille encore. Il était doux, le petit soleil. L'histoire est finie.</t>
+          <t>J'ai goûté une petite bouchée. C'était doux. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1964,7 +1972,7 @@
         <v>0.82</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.36</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2036,11 +2044,12 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Dans la cuisine, le soleil brille encore.
-enfant-f|Il était doux, le petit soleil.
+          <t>enfant-f|J'ai goûté une petite bouchée.
+enfant-f|C'était doux.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
+      <c r="AX6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2059,7 +2068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2102,6 +2111,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit captivant, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit captivant, fusion agents</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-008): histoires ≥ 3 min, plusieurs passages et leçons
Règle D17. Les 3 atomiques alimentation sont allongées : plusieurs
passages vécus, leçon d’assiette + s’asseoir à table greffées.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
+++ b/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SAN.ALI.002</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -841,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lina a faim. Une tomate rouge brille dans son assiette, comme un petit soleil. Elle en goûte une petite bouchée.</t>
+          <t>Lina a faim. Une tomate rouge brille dans son assiette, comme un petit soleil. Elle s'assoit avec maman. Elle en goûte une petite bouchée.</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lina entre dans la cuisine. Il y a du soleil. Maman est près de la table. Maman, j'ai faim ! Viens, Lina. Ton assiette est là. Lina s'assoit près de maman. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille. C'est un petit soleil ! Oui, un petit soleil. Lina se penche tout près. Ça sent le jardin. Il a quel goût ? Tu peux goûter. Une petite bouchée. Lina prend une petite bouchée. Elle goûte.</t>
+          <t>Lina pousse la porte. Elle entre dans la cuisine. Le soleil est là. Maman est près de la table. Maman, j'ai faim ! Viens, Lina. Viens t'asseoir. Lina va vers sa chaise. Elle tire un peu la chaise. Elle s'assoit près de maman. Elle pose les pieds par terre. On est ensemble. On est à table. Lina est bien assise. Sa chaise ne bouge plus. Elle écoute la cuisine. Un oiseau chante dehors. Lina sourit. Lina regarde maman. Maman sourit. Une assiette attend Lina. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille fort. C'est un petit soleil ! Oui. Un petit soleil. Lina pose les mains sur la table. Elle attend un tout petit moment. Elle regarde encore. Le soleil de la fenêtre le touche. Lina se penche tout près. Ça sent le jardin. Lina sent encore. C'est le jardin, tout près. Elle reste un moment. Lina ouvre grand les yeux. Il a quel goût ? Tu peux goûter. Une petite bouchée. Lina prend une petite bouchée. Elle goûte.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1324,21 +1329,44 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Lina entre dans la cuisine.
-narrateur|Il y a du soleil.
+          <t>narrateur|Lina pousse la porte.
+narrateur|Elle entre dans la cuisine.
+narrateur|Le soleil est là.
 narrateur|Maman est près de la table.
 enfant-f|Maman, j'ai faim !
 maman|Viens, Lina.
-maman|Ton assiette est là.
-narrateur|Lina s'assoit près de maman.
+maman|Viens t'asseoir.
+narrateur|Lina va vers sa chaise.
+narrateur|Elle tire un peu la chaise.
+narrateur|Elle s'assoit près de maman.
+narrateur|Elle pose les pieds par terre.
+maman|On est ensemble.
+maman|On est à table.
+narrateur|Lina est bien assise.
+narrateur|Sa chaise ne bouge plus.
+narrateur|Elle écoute la cuisine.
+narrateur|Un oiseau chante dehors.
+narrateur|Lina sourit.
+narrateur|Lina regarde maman.
+narrateur|Maman sourit.
+narrateur|Une assiette attend Lina.
 narrateur|Dans l'assiette, une tomate.
 narrateur|Elle est ronde.
 narrateur|Elle est rouge.
-narrateur|Elle brille.
+narrateur|Elle brille fort.
 enfant-f|C'est un petit soleil !
-maman|Oui, un petit soleil.
+maman|Oui.
+maman|Un petit soleil.
+narrateur|Lina pose les mains sur la table.
+narrateur|Elle attend un tout petit moment.
+narrateur|Elle regarde encore.
+narrateur|Le soleil de la fenêtre le touche.
 narrateur|Lina se penche tout près.
 narrateur|Ça sent le jardin.
+narrateur|Lina sent encore.
+narrateur|C'est le jardin, tout près.
+narrateur|Elle reste un moment.
+narrateur|Lina ouvre grand les yeux.
 enfant-f|Il a quel goût ?
 maman|Tu peux goûter.
 maman|Une petite bouchée.
@@ -1348,7 +1376,7 @@
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>porte,chaise</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1587,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lina mâche. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Le petit soleil est encore là.</t>
+          <t>Lina mâche. Elle mâche encore un peu. Elle est toujours assise. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Lina écoute maman. Le petit soleil est encore là.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1704,11 +1732,14 @@
       <c r="AW4" t="inlineStr">
         <is>
           <t>narrateur|Lina mâche.
+narrateur|Elle mâche encore un peu.
+narrateur|Elle est toujours assise.
 enfant-f|C'est doux, maman.
 enfant-f|Un peu sucré.
 enfant-f|Comme un soleil.
 maman|Oui.
 maman|Doux et sucré.
+narrateur|Lina écoute maman.
 narrateur|Le petit soleil est encore là.</t>
         </is>
       </c>
@@ -1737,7 +1768,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Lina boit une gorgée d'eau. Le petit soleil reste dans l'assiette. Merci, maman. Merci, Lina.</t>
+          <t>Lina reste à table. Maman verse un peu d'eau. L'eau fait un petit bruit. Lina boit une gorgée. Le petit soleil reste dans l'assiette. Lina le regarde. Il brille encore. Merci, maman. Merci, Lina. On est encore ensemble. Lina reste assise. La cuisine est calme. Lina ne se lève pas. Elle reste avec maman. Le petit soleil attend.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1873,10 +1904,21 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Lina boit une gorgée d'eau.
+          <t>narrateur|Lina reste à table.
+narrateur|Maman verse un peu d'eau.
+narrateur|L'eau fait un petit bruit.
+narrateur|Lina boit une gorgée.
 narrateur|Le petit soleil reste dans l'assiette.
+narrateur|Lina le regarde.
+narrateur|Il brille encore.
 enfant-f|Merci, maman.
-maman|Merci, Lina.</t>
+maman|Merci, Lina.
+maman|On est encore ensemble.
+narrateur|Lina reste assise.
+narrateur|La cuisine est calme.
+narrateur|Lina ne se lève pas.
+narrateur|Elle reste avec maman.
+narrateur|Le petit soleil attend.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1904,7 +1946,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai goûté une petite bouchée. C'était doux. L'histoire est finie.</t>
+          <t>J'ai goûté une petite bouchée. C'était doux. On était assises, ensemble. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2046,6 +2088,7 @@
         <is>
           <t>enfant-f|J'ai goûté une petite bouchée.
 enfant-f|C'était doux.
+maman|On était assises, ensemble.
 narrateur|L'histoire est finie.</t>
         </is>
       </c>
@@ -2068,7 +2111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2118,6 +2161,27 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit captivant, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit captivant, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit captivant, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit captivant, fusion agents</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-008): papa et maman parlent vraiment (D20)
Les adultes félicitent, discutent et posent des questions adaptées à
la scène. Le narrateur ne les remplace plus par un sourire ou « est là ».
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
+++ b/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lina pousse la porte. Elle entre dans la cuisine. Le soleil est là. Maman est près de la table. Maman, j'ai faim ! Viens, Lina. Viens t'asseoir. Lina va vers sa chaise. Elle tire un peu la chaise. Elle s'assoit près de maman. Elle pose les pieds par terre. On est ensemble. On est à table. Lina est bien assise. Sa chaise ne bouge plus. Elle écoute la cuisine. Un oiseau chante dehors. Lina sourit. Lina regarde maman. Maman sourit. Une assiette attend Lina. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille fort. C'est un petit soleil ! Oui. Un petit soleil. Lina pose les mains sur la table. Elle attend un tout petit moment. Elle regarde encore. Le soleil de la fenêtre le touche. Lina se penche tout près. Ça sent le jardin. Lina sent encore. C'est le jardin, tout près. Elle reste un moment. Lina ouvre grand les yeux. Il a quel goût ? Tu peux goûter. Une petite bouchée. Lina prend une petite bouchée. Elle goûte.</t>
+          <t>Lina pousse la porte. Elle entre dans la cuisine. Le soleil est là. Maman est près de la table. Maman, j'ai faim ! Tu as faim, Lina ? Viens t'asseoir. Lina va vers sa chaise. Elle tire un peu la chaise. Elle s'assoit près de maman. Elle pose les pieds par terre. Bravo, Lina. Tu es bien assise. On est ensemble, à table. Sa chaise ne bouge plus. Elle écoute la cuisine. Un oiseau chante dehors. Tu as entendu l'oiseau ? Oui, maman. Une assiette attend Lina. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille fort. C'est un petit soleil ! Oui. Un petit soleil. Tu as bien regardé. Lina pose les mains sur la table. Elle attend un tout petit moment. Elle regarde encore. Le soleil de la fenêtre le touche. Lina se penche tout près. Ça sent le jardin. Ça sent le jardin, hein ? Oui. Le jardin. Elle reste un moment. Lina ouvre grand les yeux. Il a quel goût ? Tu veux goûter ? Une petite bouchée. Lina prend une petite bouchée. Elle goûte.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1334,21 +1334,20 @@
 narrateur|Le soleil est là.
 narrateur|Maman est près de la table.
 enfant-f|Maman, j'ai faim !
-maman|Viens, Lina.
+maman|Tu as faim, Lina ?
 maman|Viens t'asseoir.
 narrateur|Lina va vers sa chaise.
 narrateur|Elle tire un peu la chaise.
 narrateur|Elle s'assoit près de maman.
 narrateur|Elle pose les pieds par terre.
-maman|On est ensemble.
-maman|On est à table.
-narrateur|Lina est bien assise.
+maman|Bravo, Lina.
+maman|Tu es bien assise.
+maman|On est ensemble, à table.
 narrateur|Sa chaise ne bouge plus.
 narrateur|Elle écoute la cuisine.
 narrateur|Un oiseau chante dehors.
-narrateur|Lina sourit.
-narrateur|Lina regarde maman.
-narrateur|Maman sourit.
+maman|Tu as entendu l'oiseau ?
+enfant-f|Oui, maman.
 narrateur|Une assiette attend Lina.
 narrateur|Dans l'assiette, une tomate.
 narrateur|Elle est ronde.
@@ -1357,18 +1356,19 @@
 enfant-f|C'est un petit soleil !
 maman|Oui.
 maman|Un petit soleil.
+maman|Tu as bien regardé.
 narrateur|Lina pose les mains sur la table.
 narrateur|Elle attend un tout petit moment.
 narrateur|Elle regarde encore.
 narrateur|Le soleil de la fenêtre le touche.
 narrateur|Lina se penche tout près.
 narrateur|Ça sent le jardin.
-narrateur|Lina sent encore.
-narrateur|C'est le jardin, tout près.
+maman|Ça sent le jardin, hein ?
+enfant-f|Oui. Le jardin.
 narrateur|Elle reste un moment.
 narrateur|Lina ouvre grand les yeux.
 enfant-f|Il a quel goût ?
-maman|Tu peux goûter.
+maman|Tu veux goûter ?
 maman|Une petite bouchée.
 narrateur|Lina prend une petite bouchée.
 narrateur|Elle goûte.</t>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lina mâche. Elle mâche encore un peu. Elle est toujours assise. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Lina écoute maman. Le petit soleil est encore là.</t>
+          <t>Lina mâche. Elle mâche encore un peu. Elle est toujours assise. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Bravo, Lina. Tu as goûté. C'est du bon travail. Le petit soleil est encore là. Tu as fini ta petite bouchée ?</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1737,10 +1737,12 @@
 enfant-f|C'est doux, maman.
 enfant-f|Un peu sucré.
 enfant-f|Comme un soleil.
-maman|Oui.
-maman|Doux et sucré.
-narrateur|Lina écoute maman.
-narrateur|Le petit soleil est encore là.</t>
+maman|Oui. Doux et sucré.
+maman|Bravo, Lina.
+maman|Tu as goûté.
+maman|C'est du bon travail.
+narrateur|Le petit soleil est encore là.
+maman|Tu as fini ta petite bouchée ?</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1768,7 +1770,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Lina reste à table. Maman verse un peu d'eau. L'eau fait un petit bruit. Lina boit une gorgée. Le petit soleil reste dans l'assiette. Lina le regarde. Il brille encore. Merci, maman. Merci, Lina. On est encore ensemble. Lina reste assise. La cuisine est calme. Lina ne se lève pas. Elle reste avec maman. Le petit soleil attend.</t>
+          <t>Lina reste à table. Maman verse un peu d'eau. L'eau fait un petit bruit. Tu veux un peu d'eau ? Lina boit une gorgée. Le petit soleil reste dans l'assiette. Lina le regarde. Il brille encore. Merci, maman. Merci, Lina. On reste encore un peu ensemble ? Oui. Lina reste assise. La cuisine est calme. Tu es encore bien assise. Bravo. Le petit soleil attend.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1907,17 +1909,19 @@
           <t>narrateur|Lina reste à table.
 narrateur|Maman verse un peu d'eau.
 narrateur|L'eau fait un petit bruit.
+maman|Tu veux un peu d'eau ?
 narrateur|Lina boit une gorgée.
 narrateur|Le petit soleil reste dans l'assiette.
 narrateur|Lina le regarde.
 narrateur|Il brille encore.
 enfant-f|Merci, maman.
 maman|Merci, Lina.
-maman|On est encore ensemble.
+maman|On reste encore un peu ensemble ?
+enfant-f|Oui.
 narrateur|Lina reste assise.
 narrateur|La cuisine est calme.
-narrateur|Lina ne se lève pas.
-narrateur|Elle reste avec maman.
+maman|Tu es encore bien assise.
+maman|Bravo.
 narrateur|Le petit soleil attend.</t>
         </is>
       </c>
@@ -1946,7 +1950,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai goûté une petite bouchée. C'était doux. On était assises, ensemble. L'histoire est finie.</t>
+          <t>J'ai goûté une petite bouchée. C'était doux. Bravo. Tu as fait du bon travail. On était assises, ensemble. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2088,6 +2092,8 @@
         <is>
           <t>enfant-f|J'ai goûté une petite bouchée.
 enfant-f|C'était doux.
+maman|Bravo.
+maman|Tu as fait du bon travail.
 maman|On était assises, ensemble.
 narrateur|L'histoire est finie.</t>
         </is>
@@ -2111,7 +2117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2182,6 +2188,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit captivant, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit captivant, fusion agents</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-009): trois ouvertures du monde (Sarah, Amir, Nino)
Plus de constat sec. Maison, pluie, marché, détails, puis l’action.
Amorces différentes. Audio plus tard. Les agents continuent le corpus.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
+++ b/stories/arbres/ATOM-SAN.ALI.001-01.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Lina a faim. Une tomate rouge brille dans son assiette, comme un petit soleil. Elle s'assoit avec maman. Elle en goûte une petite bouchée.</t>
+          <t>Un rayon entre dans la cuisine. Sarah a faim. Une tomate rouge brille, comme un petit soleil. Elle s'assoit avec maman. Elle en goûte une petite bouchée.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Lina pousse la porte. Elle entre dans la cuisine. Le soleil est là. Maman est près de la table. Maman, j'ai faim ! Tu as faim, Lina ? Viens t'asseoir. Lina va vers sa chaise. Elle tire un peu la chaise. Elle s'assoit près de maman. Elle pose les pieds par terre. Bravo, Lina. Tu es bien assise. On est ensemble, à table. Sa chaise ne bouge plus. Elle écoute la cuisine. Un oiseau chante dehors. Tu as entendu l'oiseau ? Oui, maman. Une assiette attend Lina. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille fort. C'est un petit soleil ! Oui. Un petit soleil. Tu as bien regardé. Lina pose les mains sur la table. Elle attend un tout petit moment. Elle regarde encore. Le soleil de la fenêtre le touche. Lina se penche tout près. Ça sent le jardin. Ça sent le jardin, hein ? Oui. Le jardin. Elle reste un moment. Lina ouvre grand les yeux. Il a quel goût ? Tu veux goûter ? Une petite bouchée. Lina prend une petite bouchée. Elle goûte.</t>
+          <t>La maison est petite. Elle est au bout d'un chemin. Le chemin sent l'herbe mouillée. Sarah vit ici, avec maman. Papa est au jardin, tout près. Ce matin, le ciel est clair. Un rayon glisse sur le carrelage. Il est chaud, tout jaune. Ça sent le pain. Sarah a le ventre qui parle. Maman, j'ai faim ! Tu as faim, Sarah ? Viens. La cuisine t'attend. Sarah pousse la porte. La porte fait un petit bruit. Maman est près de la table. Viens t'asseoir. Sarah va vers sa chaise. Elle tire un peu la chaise. Elle s'assoit près de maman. Elle pose les pieds par terre. Bravo, Sarah. Tu es bien assise. On est ensemble, à table. Sa chaise ne bouge plus. Un oiseau chante dehors. Tu as entendu l'oiseau ? Oui, maman. Une assiette attend Sarah. Dans l'assiette, une tomate. Elle est ronde. Elle est rouge. Elle brille fort. C'est un petit soleil ! Oui. Un petit soleil. Tu as bien regardé. Sarah pose les mains sur la table. Le rayon touche la tomate. Sarah se penche tout près. Ça sent le jardin. Ça sent le jardin, hein ? Oui. Le jardin. Il a quel goût ? Tu veux goûter ? Une petite bouchée. Sarah prend une petite bouchée. Elle goûte.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1329,26 +1329,35 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Lina pousse la porte.
-narrateur|Elle entre dans la cuisine.
-narrateur|Le soleil est là.
+          <t>narrateur|La maison est petite.
+narrateur|Elle est au bout d'un chemin.
+narrateur|Le chemin sent l'herbe mouillée.
+narrateur|Sarah vit ici, avec maman.
+narrateur|Papa est au jardin, tout près.
+narrateur|Ce matin, le ciel est clair.
+narrateur|Un rayon glisse sur le carrelage.
+narrateur|Il est chaud, tout jaune.
+narrateur|Ça sent le pain.
+narrateur|Sarah a le ventre qui parle.
+enfant-f|Maman, j'ai faim !
+maman|Tu as faim, Sarah ?
+maman|Viens. La cuisine t'attend.
+narrateur|Sarah pousse la porte.
+narrateur|La porte fait un petit bruit.
 narrateur|Maman est près de la table.
-enfant-f|Maman, j'ai faim !
-maman|Tu as faim, Lina ?
 maman|Viens t'asseoir.
-narrateur|Lina va vers sa chaise.
+narrateur|Sarah va vers sa chaise.
 narrateur|Elle tire un peu la chaise.
 narrateur|Elle s'assoit près de maman.
 narrateur|Elle pose les pieds par terre.
-maman|Bravo, Lina.
+maman|Bravo, Sarah.
 maman|Tu es bien assise.
 maman|On est ensemble, à table.
 narrateur|Sa chaise ne bouge plus.
-narrateur|Elle écoute la cuisine.
 narrateur|Un oiseau chante dehors.
 maman|Tu as entendu l'oiseau ?
 enfant-f|Oui, maman.
-narrateur|Une assiette attend Lina.
+narrateur|Une assiette attend Sarah.
 narrateur|Dans l'assiette, une tomate.
 narrateur|Elle est ronde.
 narrateur|Elle est rouge.
@@ -1357,20 +1366,16 @@
 maman|Oui.
 maman|Un petit soleil.
 maman|Tu as bien regardé.
-narrateur|Lina pose les mains sur la table.
-narrateur|Elle attend un tout petit moment.
-narrateur|Elle regarde encore.
-narrateur|Le soleil de la fenêtre le touche.
-narrateur|Lina se penche tout près.
+narrateur|Sarah pose les mains sur la table.
+narrateur|Le rayon touche la tomate.
+narrateur|Sarah se penche tout près.
 narrateur|Ça sent le jardin.
 maman|Ça sent le jardin, hein ?
 enfant-f|Oui. Le jardin.
-narrateur|Elle reste un moment.
-narrateur|Lina ouvre grand les yeux.
 enfant-f|Il a quel goût ?
 maman|Tu veux goûter ?
 maman|Une petite bouchée.
-narrateur|Lina prend une petite bouchée.
+narrateur|Sarah prend une petite bouchée.
 narrateur|Elle goûte.</t>
         </is>
       </c>
@@ -1403,7 +1408,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Que fait Lina ?</t>
+          <t>Que fait Sarah ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1559,7 +1564,7 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Que fait Lina ?</t>
+          <t>narrateur|Que fait Sarah ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1587,7 +1592,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Lina mâche. Elle mâche encore un peu. Elle est toujours assise. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Bravo, Lina. Tu as goûté. C'est du bon travail. Le petit soleil est encore là. Tu as fini ta petite bouchée ?</t>
+          <t>Sarah mâche. Elle mâche encore un peu. Elle est toujours assise. C'est doux, maman. Un peu sucré. Comme un soleil. Oui. Doux et sucré. Bravo, Sarah. Tu as goûté. C'est du bon travail. Le petit soleil est encore là. Tu as fini ta petite bouchée ?</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1731,14 +1736,14 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Lina mâche.
+          <t>narrateur|Sarah mâche.
 narrateur|Elle mâche encore un peu.
 narrateur|Elle est toujours assise.
 enfant-f|C'est doux, maman.
 enfant-f|Un peu sucré.
 enfant-f|Comme un soleil.
 maman|Oui. Doux et sucré.
-maman|Bravo, Lina.
+maman|Bravo, Sarah.
 maman|Tu as goûté.
 maman|C'est du bon travail.
 narrateur|Le petit soleil est encore là.
@@ -1770,7 +1775,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Lina reste à table. Maman verse un peu d'eau. L'eau fait un petit bruit. Tu veux un peu d'eau ? Lina boit une gorgée. Le petit soleil reste dans l'assiette. Lina le regarde. Il brille encore. Merci, maman. Merci, Lina. On reste encore un peu ensemble ? Oui. Lina reste assise. La cuisine est calme. Tu es encore bien assise. Bravo. Le petit soleil attend.</t>
+          <t>Sarah reste à table. Maman verse un peu d'eau. L'eau fait un petit bruit. Tu veux un peu d'eau ? Sarah boit une gorgée. Le petit soleil reste dans l'assiette. Sarah le regarde. Il brille encore. Merci, maman. Merci, Sarah. On reste encore un peu ensemble ? Oui. Sarah reste assise. La cuisine est calme. Tu es encore bien assise. Bravo. Le petit soleil attend.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1906,19 +1911,19 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Lina reste à table.
+          <t>narrateur|Sarah reste à table.
 narrateur|Maman verse un peu d'eau.
 narrateur|L'eau fait un petit bruit.
 maman|Tu veux un peu d'eau ?
-narrateur|Lina boit une gorgée.
+narrateur|Sarah boit une gorgée.
 narrateur|Le petit soleil reste dans l'assiette.
-narrateur|Lina le regarde.
+narrateur|Sarah le regarde.
 narrateur|Il brille encore.
 enfant-f|Merci, maman.
-maman|Merci, Lina.
+maman|Merci, Sarah.
 maman|On reste encore un peu ensemble ?
 enfant-f|Oui.
-narrateur|Lina reste assise.
+narrateur|Sarah reste assise.
 narrateur|La cuisine est calme.
 maman|Tu es encore bien assise.
 maman|Bravo.
@@ -2117,7 +2122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2197,6 +2202,13 @@
       <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit captivant, fusion agents</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>